<commit_message>
Scrub personal info from runbook and verification workbooks
Replaced 6 occurrences across 2 XLSX files:
- prabhurao5@gmail.com -> admin@example.com
- 98dc1d22-13a3-49f3-8e33-ad1546784a08 -> <your-admin-user-id>

Plan workbook had no hits; SQL/TSX/Edge Function files were already clean.
Repo can now be made public without leaking personal identifiers.

Co-Authored-By: Claude Opus 4.7 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/phase-b-rollout-runbook.xlsx
+++ b/phase-b-rollout-runbook.xlsx
@@ -542,6 +542,7 @@
         </is>
       </c>
     </row>
+    <row r="2"/>
     <row r="3" ht="26" customHeight="1">
       <c r="A3" s="2" t="inlineStr">
         <is>
@@ -634,6 +635,7 @@
       <c r="C9" s="4" t="n"/>
     </row>
     <row r="10" ht="26" customHeight="1"/>
+    <row r="11"/>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="5" t="inlineStr">
         <is>
@@ -671,7 +673,7 @@
     <row r="16" ht="50" customHeight="1">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>☐ Verify your prabhurao5@gmail.com account is currently the only admin in org_members for Demo Hospital. If you accidentally lose admin access mid-migration (the change_member_role guards prevent self-demotion, but accidents happen), you'll need DB-direct access to recover.</t>
+          <t>☐ Verify your admin@example.com account is currently the only admin in org_members for Demo Hospital. If you accidentally lose admin access mid-migration (the change_member_role guards prevent self-demotion, but accidents happen), you'll need DB-direct access to recover.</t>
         </is>
       </c>
       <c r="B16" s="6" t="n"/>
@@ -1740,7 +1742,7 @@
       </c>
       <c r="C5" s="8" t="inlineStr">
         <is>
-          <t>From a session signed in as you (prabhurao5@gmail.com):
+          <t>From a session signed in as you (admin@example.com):
 SELECT private.accept_org_invite('&lt;token&gt;');</t>
         </is>
       </c>

</xml_diff>